<commit_message>
fix: Fix broken Excel file - unicode escapes and chart XML
- Fixed \u20ac (euro sign) → actual € character in chart XML
- Fixed \u00e4 (ä) → actual ä in month names (März)
- XML was syntactically valid but Excel couldn't parse JS escapes
- Verified with openpyxl: 2 charts detected, all 6 sheets valid
- Verified with xmllint: all chart/drawing XML well-formed
- Verified with ExcelJS: file reads back correctly

https://claude.ai/code/session_01MhbCMEQuVFuGKkcRvxCBuV
</commit_message>
<xml_diff>
--- a/budget-tracker/Budget-Tracker.xlsx
+++ b/budget-tracker/Budget-Tracker.xlsx
@@ -1509,7 +1509,7 @@
             <c:numRef>
               <c:f>Dashboard!$C$39:$C$46</c:f>
               <c:numCache>
-                <c:formatCode>#,##0.00\ "\u20ac"</c:formatCode>
+                <c:formatCode>#,##0.00\ "€"</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
@@ -1674,7 +1674,7 @@
                   <c:v>Feb</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>M\u00e4r</c:v>
+                  <c:v>Mär</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>Apr</c:v>
@@ -1710,7 +1710,7 @@
             <c:numRef>
               <c:f>Dashboard!$C$13:$C$24</c:f>
               <c:numCache>
-                <c:formatCode>#,##0.00\ "\u20ac"</c:formatCode>
+                <c:formatCode>#,##0.00\ "€"</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
@@ -1787,7 +1787,7 @@
                   <c:v>Feb</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>M\u00e4r</c:v>
+                  <c:v>Mär</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>Apr</c:v>
@@ -1823,7 +1823,7 @@
             <c:numRef>
               <c:f>Dashboard!$D$13:$D$24</c:f>
               <c:numCache>
-                <c:formatCode>#,##0.00\ "\u20ac"</c:formatCode>
+                <c:formatCode>#,##0.00\ "€"</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
@@ -1916,7 +1916,7 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:numFmt formatCode="#,##0\ &quot;\u20ac&quot;" sourceLinked="0"/>
+        <c:numFmt formatCode="#,##0\ &quot;€&quot;" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>

</xml_diff>